<commit_message>
Update robot assets and document CAD navigation
</commit_message>
<xml_diff>
--- a/1_RobotModelSelect/Robot_model.xlsx
+++ b/1_RobotModelSelect/Robot_model.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCARA Robot" sheetId="1" r:id="R7fee3f2713174efe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6-Axis Robot" sheetId="2" r:id="R03ba95a2e12d49d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accessories" sheetId="3" r:id="Raeda937511494918"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expansion Card" sheetId="4" r:id="Ra85408ed6f6d446e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCARA Robot" sheetId="1" r:id="R5dd4076d56744eb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6-Axis Robot" sheetId="2" r:id="Rb3e444c5578e40fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accessories" sheetId="3" r:id="R0bd0187c93fe46bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expansion Card" sheetId="4" r:id="R37272a3d39b84222"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1217,9 +1217,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -8173,6 +8173,9 @@
       <x:c r="F1" s="4" t="s">
         <x:v>111</x:v>
       </x:c>
+      <x:c r="G1" t="str">
+        <x:v>Set ID</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A2" s="13" t="s">
@@ -8193,6 +8196,7 @@
       <x:c r="F2" s="3" t="s">
         <x:v>117</x:v>
       </x:c>
+      <x:c r="G2"/>
     </x:row>
     <x:row r="3" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A3" s="13" t="s">
@@ -8213,6 +8217,7 @@
       <x:c r="F3" s="3" t="s">
         <x:v>120</x:v>
       </x:c>
+      <x:c r="G3"/>
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A4" s="13" t="s">
@@ -8233,6 +8238,7 @@
       <x:c r="F4" s="3" t="s">
         <x:v>120</x:v>
       </x:c>
+      <x:c r="G4"/>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A5" s="13" t="s">
@@ -8253,6 +8259,7 @@
       <x:c r="F5" s="3" t="s">
         <x:v>124</x:v>
       </x:c>
+      <x:c r="G5"/>
     </x:row>
     <x:row r="6" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A6" s="13" t="s">
@@ -8273,6 +8280,7 @@
       <x:c r="F6" s="3" t="s">
         <x:v>124</x:v>
       </x:c>
+      <x:c r="G6"/>
     </x:row>
     <x:row r="7" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A7" s="13" t="s">
@@ -8293,6 +8301,7 @@
       <x:c r="F7" s="3" t="s">
         <x:v>128</x:v>
       </x:c>
+      <x:c r="G7"/>
     </x:row>
     <x:row r="8" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A8" s="13" t="s">
@@ -8313,6 +8322,7 @@
       <x:c r="F8" s="3" t="s">
         <x:v>131</x:v>
       </x:c>
+      <x:c r="G8"/>
     </x:row>
     <x:row r="9" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A9" s="13" t="s">
@@ -8333,6 +8343,7 @@
       <x:c r="F9" s="3" t="s">
         <x:v>131</x:v>
       </x:c>
+      <x:c r="G9"/>
     </x:row>
     <x:row r="10" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A10" s="13" t="s">
@@ -8353,6 +8364,7 @@
       <x:c r="F10" s="3" t="s">
         <x:v>131</x:v>
       </x:c>
+      <x:c r="G10"/>
     </x:row>
     <x:row r="11" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A11" s="13" t="s">
@@ -8373,6 +8385,7 @@
       <x:c r="F11" s="3" t="s">
         <x:v>136</x:v>
       </x:c>
+      <x:c r="G11"/>
     </x:row>
     <x:row r="12" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A12" s="13" t="s">
@@ -8393,6 +8406,7 @@
       <x:c r="F12" s="3" t="s">
         <x:v>136</x:v>
       </x:c>
+      <x:c r="G12"/>
     </x:row>
     <x:row r="13" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A13" s="13" t="s">
@@ -8413,6 +8427,7 @@
       <x:c r="F13" s="3" t="s">
         <x:v>139</x:v>
       </x:c>
+      <x:c r="G13"/>
     </x:row>
     <x:row r="14" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A14" s="13" t="s">
@@ -8433,6 +8448,7 @@
       <x:c r="F14" s="3" t="s">
         <x:v>142</x:v>
       </x:c>
+      <x:c r="G14"/>
     </x:row>
     <x:row r="15" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A15" s="13" t="s">
@@ -8453,6 +8469,7 @@
       <x:c r="F15" s="3" t="s">
         <x:v>144</x:v>
       </x:c>
+      <x:c r="G15"/>
     </x:row>
     <x:row r="16" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A16" s="13" t="s">
@@ -8473,6 +8490,7 @@
       <x:c r="F16" s="3" t="s">
         <x:v>144</x:v>
       </x:c>
+      <x:c r="G16"/>
     </x:row>
     <x:row r="17" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A17" s="13" t="s">
@@ -8493,6 +8511,7 @@
       <x:c r="F17" s="3" t="s">
         <x:v>144</x:v>
       </x:c>
+      <x:c r="G17"/>
     </x:row>
     <x:row r="18" ht="16.5" customHeight="1">
       <x:c r="A18" s="3" t="s">
@@ -8513,6 +8532,7 @@
       <x:c r="F18" s="3" t="s">
         <x:v>149</x:v>
       </x:c>
+      <x:c r="G18"/>
     </x:row>
     <x:row r="19" ht="16.5" customHeight="1">
       <x:c r="A19" s="3" t="s">
@@ -8533,6 +8553,7 @@
       <x:c r="F19" s="3" t="s">
         <x:v>153</x:v>
       </x:c>
+      <x:c r="G19"/>
     </x:row>
     <x:row r="20" ht="16.5" customHeight="1">
       <x:c r="A20" s="3" t="s">
@@ -8553,6 +8574,7 @@
       <x:c r="F20" s="3" t="s">
         <x:v>158</x:v>
       </x:c>
+      <x:c r="G20"/>
     </x:row>
     <x:row r="21" ht="16.5" customHeight="1">
       <x:c r="A21" s="3" t="s">
@@ -8573,6 +8595,7 @@
       <x:c r="F21" s="3" t="s">
         <x:v>158</x:v>
       </x:c>
+      <x:c r="G21"/>
     </x:row>
     <x:row r="22" ht="16.5" customHeight="1">
       <x:c r="A22" s="3" t="s">
@@ -8593,6 +8616,7 @@
       <x:c r="F22" s="3" t="s">
         <x:v>158</x:v>
       </x:c>
+      <x:c r="G22"/>
     </x:row>
     <x:row r="23" ht="16.5" customHeight="1">
       <x:c r="A23" s="3" t="s">
@@ -8613,6 +8637,7 @@
       <x:c r="F23" s="3" t="s">
         <x:v>166</x:v>
       </x:c>
+      <x:c r="G23"/>
     </x:row>
     <x:row r="24" ht="16.5" customHeight="1">
       <x:c r="A24" s="3" t="s">
@@ -8633,6 +8658,7 @@
       <x:c r="F24" s="3" t="s">
         <x:v>166</x:v>
       </x:c>
+      <x:c r="G24"/>
     </x:row>
     <x:row r="25" ht="16.5" customHeight="1">
       <x:c r="A25" s="3" t="s">
@@ -8653,6 +8679,7 @@
       <x:c r="F25" s="3" t="s">
         <x:v>172</x:v>
       </x:c>
+      <x:c r="G25"/>
     </x:row>
     <x:row r="26" ht="16.5" customHeight="1">
       <x:c r="A26" s="3" t="s">
@@ -8673,6 +8700,7 @@
       <x:c r="F26" s="3" t="s">
         <x:v>172</x:v>
       </x:c>
+      <x:c r="G26"/>
     </x:row>
     <x:row r="27" ht="16.5" customHeight="1">
       <x:c r="A27" s="3" t="s">
@@ -8693,6 +8721,7 @@
       <x:c r="F27" s="3" t="s">
         <x:v>172</x:v>
       </x:c>
+      <x:c r="G27"/>
     </x:row>
     <x:row r="28" ht="16.5" customHeight="1">
       <x:c r="A28" s="3" t="s">
@@ -8713,6 +8742,7 @@
       <x:c r="F28" s="3" t="s">
         <x:v>172</x:v>
       </x:c>
+      <x:c r="G28"/>
     </x:row>
     <x:row r="29" ht="16.5" customHeight="1">
       <x:c r="A29" s="13" t="s">
@@ -8733,6 +8763,7 @@
       <x:c r="F29" s="3" t="s">
         <x:v>183</x:v>
       </x:c>
+      <x:c r="G29"/>
     </x:row>
     <x:row r="30" ht="16.5" customHeight="1">
       <x:c r="A30" s="13" t="s">
@@ -8753,6 +8784,7 @@
       <x:c r="F30" s="3" t="s">
         <x:v>183</x:v>
       </x:c>
+      <x:c r="G30"/>
     </x:row>
     <x:row r="31" ht="16.5" customHeight="1">
       <x:c r="A31" s="13" t="s">
@@ -8773,6 +8805,7 @@
       <x:c r="F31" s="3" t="s">
         <x:v>183</x:v>
       </x:c>
+      <x:c r="G31"/>
     </x:row>
     <x:row r="32" ht="16.5" customHeight="1">
       <x:c r="A32" s="3" t="s">
@@ -8793,6 +8826,7 @@
       <x:c r="F32" s="3" t="s">
         <x:v>190</x:v>
       </x:c>
+      <x:c r="G32"/>
     </x:row>
     <x:row r="33" ht="16.5" customHeight="1">
       <x:c r="A33" s="3" t="s">
@@ -8813,6 +8847,7 @@
       <x:c r="F33" s="3" t="s">
         <x:v>191</x:v>
       </x:c>
+      <x:c r="G33"/>
     </x:row>
     <x:row r="34" ht="16.5" customHeight="1">
       <x:c r="A34" s="24" t="s">
@@ -8833,6 +8868,7 @@
       <x:c r="F34" s="24" t="s">
         <x:v>196</x:v>
       </x:c>
+      <x:c r="G34"/>
     </x:row>
     <x:row r="35" ht="16.5" customHeight="1">
       <x:c r="A35" s="3" t="s">
@@ -8853,6 +8889,7 @@
       <x:c r="F35" s="3" t="s">
         <x:v>201</x:v>
       </x:c>
+      <x:c r="G35"/>
     </x:row>
     <x:row r="36" ht="16.5" customHeight="1">
       <x:c r="A36" s="3" t="s">
@@ -8873,6 +8910,7 @@
       <x:c r="F36" s="3" t="s">
         <x:v>204</x:v>
       </x:c>
+      <x:c r="G36"/>
     </x:row>
     <x:row r="37" ht="16.5" customHeight="1">
       <x:c r="A37" s="3" t="s">
@@ -8893,6 +8931,7 @@
       <x:c r="F37" s="3" t="s">
         <x:v>207</x:v>
       </x:c>
+      <x:c r="G37"/>
     </x:row>
     <x:row r="38" ht="16.5" customHeight="1">
       <x:c r="A38" s="3" t="s">
@@ -8913,6 +8952,7 @@
       <x:c r="F38" s="3" t="s">
         <x:v>209</x:v>
       </x:c>
+      <x:c r="G38"/>
     </x:row>
     <x:row r="39" s="1" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A39" s="3" t="s">
@@ -8933,6 +8973,7 @@
       <x:c r="F39" s="3" t="s">
         <x:v>213</x:v>
       </x:c>
+      <x:c r="G39"/>
     </x:row>
     <x:row r="40" ht="16.5" customHeight="1">
       <x:c r="A40" s="3" t="s">
@@ -8953,6 +8994,7 @@
       <x:c r="F40" s="3" t="s">
         <x:v>216</x:v>
       </x:c>
+      <x:c r="G40"/>
     </x:row>
     <x:row r="41" ht="16.5" customHeight="1">
       <x:c r="A41" s="3" t="s">
@@ -8972,6 +9014,99 @@
       </x:c>
       <x:c r="F41" s="3" t="s">
         <x:v>220</x:v>
+      </x:c>
+      <x:c r="G41"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
+        <x:v>Cable &amp; Connector</x:v>
+      </x:c>
+      <x:c r="B42" t="str">
+        <x:v>Robot arm I/O cable</x:v>
+      </x:c>
+      <x:c r="C42" t="str">
+        <x:v>1504UP81</x:v>
+      </x:c>
+      <x:c r="D42" t="str">
+        <x:v>2m</x:v>
+      </x:c>
+      <x:c r="E42" t="str">
+        <x:v>R15H, R20H</x:v>
+      </x:c>
+      <x:c r="F42" t="str">
+        <x:v>26 pin connector cable</x:v>
+      </x:c>
+      <x:c r="G42" t="str">
+        <x:v>R15H-R20H-1504UP81</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="str">
+        <x:v>Cable &amp; Connector</x:v>
+      </x:c>
+      <x:c r="B43" t="str">
+        <x:v>Robot Body I/O cable</x:v>
+      </x:c>
+      <x:c r="C43" t="str">
+        <x:v>1504UP81</x:v>
+      </x:c>
+      <x:c r="D43" t="str">
+        <x:v>7m</x:v>
+      </x:c>
+      <x:c r="E43" t="str">
+        <x:v>R15H, R20H</x:v>
+      </x:c>
+      <x:c r="F43" t="str">
+        <x:v>26 pin cable</x:v>
+      </x:c>
+      <x:c r="G43" t="str">
+        <x:v>R15H-R20H-1504UP81</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>Connector</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>Robot arm I/O cable</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>1504CU41</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>R15H, R20H</x:v>
+      </x:c>
+      <x:c r="F44" t="str">
+        <x:v>26 pin connector only</x:v>
+      </x:c>
+      <x:c r="G44" t="str">
+        <x:v>R15H-R20H-1504CU41</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>Cable &amp; Connector</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>Robot Body I/O cable</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>1504CU41</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>7m</x:v>
+      </x:c>
+      <x:c r="E45" t="str">
+        <x:v>R15H, R20H</x:v>
+      </x:c>
+      <x:c r="F45" t="str">
+        <x:v>26 pin cable</x:v>
+      </x:c>
+      <x:c r="G45" t="str">
+        <x:v>R15H-R20H-1504CU41</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>